<commit_message>
docs(navis): comptes de service dedies par usage, pas un n4api partage
L'Universal Query API ne voit que les filtres crees par le compte qui
les a enregistres : un compte partage entre plusieurs integrations
empecherait de couper l'acces de l'une sans couper les autres. Ajoute
la recommandation d'un compte de service dedie au chatbot (ex.
n4api-chatbot) dans le doc et une petite table de comptes de service
dans le classeur, en plus des coordonnees serveur/portee deja
presentes.
</commit_message>
<xml_diff>
--- a/docs/99-filtres-navis-a-creer.xlsx
+++ b/docs/99-filtres-navis-a-creer.xlsx
@@ -619,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -680,33 +680,25 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Compte de service (role n4api)</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Nom d'utilisateur</t>
-        </is>
-      </c>
+          <t>operatorId</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr"/>
       <c r="C6" s="8" t="inlineStr"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Mot de passe du compte de service</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>A transmettre par un canal securise, jamais par email/chat</t>
-        </is>
-      </c>
+          <t>complexId</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr"/>
       <c r="C7" s="8" t="inlineStr"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>operatorId</t>
+          <t>facilityId</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr"/>
@@ -715,33 +707,72 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>complexId</t>
+          <t>yardId</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr"/>
       <c r="C9" s="8" t="inlineStr"/>
     </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>facilityId</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr"/>
-      <c r="C10" s="8" t="inlineStr"/>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>yardId</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr"/>
-      <c r="C11" s="8" t="inlineStr"/>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Comptes de service (un par usage — voir note)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="70" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>L'Universal Query API ne voit que les filtres crees par le compte qui les a enregistres. Un compte partage entre plusieurs integrations empeche de couper l'acces de l'une sans couper les autres, et melange leur historique d'audit. Prevoir un compte de service dedie par usage (ex. n4api-chatbot pour ce projet), distinct de tout autre compte deja utilise ou a venir. TOUS les filtres du chatbot doivent etre crees en etant connecte avec ce meme compte, jamais avec un compte personnel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Nom du compte</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Usage / integration</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Filtres qu'il doit voir</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>n4api-chatbot</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr"/>
+      <c r="C15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="8" t="inlineStr"/>
+      <c r="B16" s="8" t="inlineStr"/>
+      <c r="C16" s="8" t="inlineStr"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="8" t="inlineStr"/>
+      <c r="B17" s="8" t="inlineStr"/>
+      <c r="C17" s="8" t="inlineStr"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="8" t="inlineStr"/>
+      <c r="B18" s="8" t="inlineStr"/>
+      <c r="C18" s="8" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A12:C12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(navis): reconciliation avec les 30 categories reelles de requetes (REQUETE VBS.xlsx)
Ajoute 5 filtres (8 -> 13) deduits des vraies categories fournies par
CIT : APPOINTMENT_STATUS (VBS - rendez-vous/creneaux, confirme lie a
Navis), UNIT_VGM_STATUS, EDI_MESSAGE_STATUS (COPARN), TRANSPORT_ORDER_STATUS
(mission/assignation), TERMINAL_TRANSFER_STATUS (HINO/CIT). Etend le
filtre #1 avec le statut dangereux/IMDG. Ajoute une feuille de
correspondance categorie reelle -> source (Navis / YABA / hors
perimetre-escalade humaine), et clarifie que les 3 items OMNIO
(creation/activation/anomalie de compte) restent ambigus : ce sont des
actions d'ecriture, hors du champ strictement lecture seule de
l'Universal Query API.
</commit_message>
<xml_diff>
--- a/docs/99-filtres-navis-a-creer.xlsx
+++ b/docs/99-filtres-navis-a-creer.xlsx
@@ -10,10 +10,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Garde" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acces serveur &amp; portee" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Filtres a creer" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hors perimetre" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correspondance FAQ reelle" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hors perimetre" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Filtres a creer'!$A$1:$L$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Filtres a creer'!$A$1:$L$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Correspondance FAQ reelle'!$A$4:$C$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,8 +58,14 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="005B6472"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -99,6 +107,11 @@
         <fgColor rgb="00F3F6FB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7F7EF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -126,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -163,6 +176,16 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -784,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1215,10 +1238,230 @@
       <c r="K9" s="11" t="n"/>
       <c r="L9" s="11" t="n"/>
     </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>APPOINTMENT_STATUS</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Ecran de rendez-vous/appointments du Gate (VBS)</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Numero de conteneur, ou reference de rendez-vous, ou immatriculation camion</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Reference du rendez-vous, Creneau (date/heure), Statut (confirme/annule/realise), Type d'operation (pickup/drop-off), Conteneur associe</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Prise de rendez-vous / Annulation rendez-vous / Demande de creneau disponible / Indisponibilite VBS</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="n"/>
+      <c r="I10" s="11" t="n"/>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>A faire</t>
+        </is>
+      </c>
+      <c r="K10" s="11" t="n"/>
+      <c r="L10" s="11" t="n"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>UNIT_VGM_STATUS</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Units, colonnes VGM</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Numero de conteneur</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Numero conteneur, VGM recu (oui/non), Poids VGM, Date de reception, Methode de pesee si tracee</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Probleme VGM</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="n"/>
+      <c r="I11" s="11" t="n"/>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>A faire</t>
+        </is>
+      </c>
+      <c r="K11" s="11" t="n"/>
+      <c r="L11" s="11" t="n"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>EDI_MESSAGE_STATUS</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Vue des messages EDI entrants (a confirmer si exposee en table)</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Numero de BL ou de booking</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Type de message (COPARN...), Date de reception, Statut (recu/rejete/en attente), Motif de rejet le cas echeant</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>COPARN recu/non recu</t>
+        </is>
+      </c>
+      <c r="H12" s="11" t="n"/>
+      <c r="I12" s="11" t="n"/>
+      <c r="J12" s="7" t="inlineStr">
+        <is>
+          <t>A faire</t>
+        </is>
+      </c>
+      <c r="K12" s="11" t="n"/>
+      <c r="L12" s="11" t="n"/>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>TRANSPORT_ORDER_STATUS</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Transport Order (ASC Automated Equipment Database Interface)</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Numero de conteneur, ou reference de mission</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Reference mission, Type (pickup/dropoff/move), Statut (en attente/en cours/terminee/annulee), Equipement assigne</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Mission conteneurs / Annulation mission / Assignation</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="n"/>
+      <c r="I13" s="11" t="n"/>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>A faire</t>
+        </is>
+      </c>
+      <c r="K13" s="11" t="n"/>
+      <c r="L13" s="11" t="n"/>
+    </row>
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>TERMINAL_TRANSFER_STATUS</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>Basse-Moyenne</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>A confirmer selon modelisation du transfert HINO/CIT</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Numero de conteneur</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Statut du transfert, Site d'origine, Site de destination, Date</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Transfert conteneur HINO/CIT</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="n"/>
+      <c r="I14" s="11" t="n"/>
+      <c r="J14" s="7" t="inlineStr">
+        <is>
+          <t>A faire</t>
+        </is>
+      </c>
+      <c r="K14" s="11" t="n"/>
+      <c r="L14" s="11" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L9"/>
+  <autoFilter ref="A1:L14"/>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"A faire,En cours,Cree,Teste OK,Bloque"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1232,7 +1475,572 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Correspondance categories reelles -&gt; source de donnees</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>Source : REQUETE VBS.xlsx fourni par CIT (30 categories de requetes frequentes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Categorie reelle (FAQ)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Source proposee</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Filtre</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Statut conteneurs</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>#1 UNIT_STATUS_BY_NUMBER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>TC Introuvable</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>#1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Position Conteneurs</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>#1 / #7</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>TC innaccesible</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Navis (hold)</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>#2 UNIT_HOLDS_BY_NUMBER</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Debarquement conteneur dangereux</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Navis (statut + IMDG)</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>#1, colonnes etendues</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>Visibilite BL sur OMNIO</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Navis (OMNIO reflete Navis)</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>#3 UNITS_BY_BL_NUMBER</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>Nomination</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>#4 UNITS_BY_BOOKING_NUMBER</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Situation Navire CIT</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>#5 VESSEL_VISIT_BY_VOYAGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Attente au chargement</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Navis (gate)</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>#6 GATE_TRANSACTIONS_BY_UNIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Embouteillage Sortie</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Navis (gate), si trace</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>#6</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>Assignation</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>Navis (gate/mission)</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>#6 ou #12</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Prise de rendez vous</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Navis (VBS)</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>#9 APPOINTMENT_STATUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Annulation rendez vous</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Navis (VBS)</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>#9</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Demande de creneau disponible</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Navis (VBS)</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>#9</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Indisponibilite VBS</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Navis (VBS) - a confirmer</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t>#9</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>Probleme VGM</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>#10 UNIT_VGM_STATUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>COPARN recu/non recu</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Navis (EDI)</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="inlineStr">
+        <is>
+          <t>#11 EDI_MESSAGE_STATUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>Mission conteneurs</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Navis (transport order)</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="inlineStr">
+        <is>
+          <t>#12 TRANSPORT_ORDER_STATUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>Annulation mission</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Navis (transport order)</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="inlineStr">
+        <is>
+          <t>#12</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>Transfert conteneur HINO/CIT</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Navis, si trace</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="inlineStr">
+        <is>
+          <t>#13 TERMINAL_TRANSFER_STATUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>Creation Compte OMNIO</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>AMBIGU - action d'ecriture, pas une donnee a lire</t>
+        </is>
+      </c>
+      <c r="C25" s="21" t="inlineStr">
+        <is>
+          <t>A clarifier - voir note</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>Activation compte OMNIO</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>AMBIGU - idem</t>
+        </is>
+      </c>
+      <c r="C26" s="21" t="inlineStr">
+        <is>
+          <t>A clarifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="20" t="inlineStr">
+        <is>
+          <t>Anomalie OMNIO</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>AMBIGU - probablement incident technique</t>
+        </is>
+      </c>
+      <c r="C27" s="21" t="inlineStr">
+        <is>
+          <t>A clarifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="22" t="inlineStr">
+        <is>
+          <t>Autorisation acces BL IES</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>Cote YABA (module IES)</t>
+        </is>
+      </c>
+      <c r="C28" s="23" t="inlineStr">
+        <is>
+          <t>Hors Navis</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="22" t="inlineStr">
+        <is>
+          <t>Actualisation BADT</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>Cote YABA (deja dans le ticket YABA, IMP-14)</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="inlineStr">
+        <is>
+          <t>Hors Navis</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="22" t="inlineStr">
+        <is>
+          <t>BADT expire</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>Cote YABA</t>
+        </is>
+      </c>
+      <c r="C30" s="23" t="inlineStr">
+        <is>
+          <t>Hors Navis</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>Impression BEE</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>Cote YABA (deja dans le ticket YABA, EXP-03)</t>
+        </is>
+      </c>
+      <c r="C31" s="23" t="inlineStr">
+        <is>
+          <t>Hors Navis</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="22" t="inlineStr">
+        <is>
+          <t>RTG en panne</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Incident operationnel/equipement</t>
+        </is>
+      </c>
+      <c r="C32" s="23" t="inlineStr">
+        <is>
+          <t>Hors perimetre - escalade humaine</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="22" t="inlineStr">
+        <is>
+          <t>Probleme de reseau</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Incident IT</t>
+        </is>
+      </c>
+      <c r="C33" s="23" t="inlineStr">
+        <is>
+          <t>Hors perimetre - escalade humaine</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="24" customHeight="1">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>Autre</t>
+        </is>
+      </c>
+      <c r="B34" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C34" s="19" t="inlineStr">
+        <is>
+          <t>Toujours escalade humaine (IA-03)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:C34"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1247,7 +2055,7 @@
       </c>
     </row>
     <row r="3" ht="50" customHeight="1">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="24" t="inlineStr">
         <is>
           <t>Facturation / paiement</t>
         </is>
@@ -1259,14 +2067,38 @@
       </c>
     </row>
     <row r="4" ht="50" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
-        <is>
-          <t>Toute action en ecriture (holds, confirmations...)</t>
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>Toute action en ecriture (holds, confirmations, creation/activation de compte...)</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
           <t>L'Universal Query API est strictement en lecture seule par conception. Toute action reelle reste hors perimetre du chatbot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="50" customHeight="1">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>BADT / BEE (actualisation, expiration, impression)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Ces documents sont deja deposes dans le ticket YABA par le Pilote Controle Documentaire (IMP-14, EXP-03). Le chatbot doit lire l'etat du ticket YABA, pas interroger Navis pour ca.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="50" customHeight="1">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>RTG en panne, Probleme de reseau</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Incidents operationnels/IT, pas des questions sur un conteneur ou un dossier. A escalader directement vers le support humain (IA-03, IA-06).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(navis): colonne Application (Navis/OMNIO) + verdict lecture seule pour les 3 items OMNIO
Ajoute une colonne "Application" a chaque filtre et a la correspondance
FAQ (Navis / OMNIO / YABA). Tranche explicitement les 3 categories
OMNIO (creation, activation, anomalie de compte) en "Aucune (lecture
impossible)" : deux sont des actions d'ecriture, une est un
signalement d'incident - aucune des deux ne peut etre servie par une
requete en lecture seule, quelle que soit l'application visee. Precise
que "annulation rendez-vous"/"annulation mission" ne peuvent au mieux
que LIRE le statut annule, jamais executer l'annulation elle-meme.
</commit_message>
<xml_diff>
--- a/docs/99-filtres-navis-a-creer.xlsx
+++ b/docs/99-filtres-navis-a-creer.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hors perimetre" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Filtres a creer'!$A$1:$L$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Correspondance FAQ reelle'!$A$4:$C$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Filtres a creer'!$A$1:$M$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Correspondance FAQ reelle'!$A$4:$D$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -139,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -184,6 +184,8 @@
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -807,21 +809,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -832,55 +835,60 @@
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
           <t>Nom du filtre (propose)</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Priorite</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Ecran N4 source</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Parametre attendu</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Colonnes a inclure</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Question client couverte</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>Nom reel enregistre (si different)</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>Nom reel du champ parametre</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>Date de creation</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
+      <c r="M1" s="5" t="inlineStr">
         <is>
           <t>Commentaire / testeur</t>
         </is>
@@ -892,43 +900,48 @@
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
           <t>UNIT_STATUS_BY_NUMBER</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>Units (Yard / Equipment)</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Numero de conteneur (UNIT_NBR ou equivalent)</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>Numero conteneur, Statut/Category, Emplacement (bloc/rangee/niveau), Navire, Voyage, Sens (Import/Export), Date de dechargement (ou gate-in export), Ligne maritime</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>Ou est mon conteneur ? / Est-il decharge ?</t>
         </is>
       </c>
-      <c r="H2" s="11" t="n"/>
       <c r="I2" s="11" t="n"/>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="J2" s="11" t="n"/>
+      <c r="K2" s="7" t="inlineStr">
         <is>
           <t>A faire</t>
         </is>
       </c>
-      <c r="K2" s="11" t="n"/>
       <c r="L2" s="11" t="n"/>
+      <c r="M2" s="11" t="n"/>
     </row>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="7" t="n">
@@ -936,43 +949,48 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
           <t>UNIT_HOLDS_BY_NUMBER</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>Units &gt; onglet Holds (ou vue Holds dediee)</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>Numero de conteneur</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>Numero conteneur, Type de hold (douane, facturation, ligne...), Statut du hold (actif/leve), Raison, Date de pose</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>Pourquoi je ne peux pas recuperer mon conteneur ?</t>
         </is>
       </c>
-      <c r="H3" s="11" t="n"/>
       <c r="I3" s="11" t="n"/>
-      <c r="J3" s="7" t="inlineStr">
+      <c r="J3" s="11" t="n"/>
+      <c r="K3" s="7" t="inlineStr">
         <is>
           <t>A faire</t>
         </is>
       </c>
-      <c r="K3" s="11" t="n"/>
       <c r="L3" s="11" t="n"/>
+      <c r="M3" s="11" t="n"/>
     </row>
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="7" t="n">
@@ -980,43 +998,48 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
           <t>UNITS_BY_BL_NUMBER</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>Units, filtre sur le champ BL</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Numero de BL</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>Numero conteneur, Statut, Emplacement, Poids, Taille/Type</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>Quels conteneurs sont sur mon BL X ?</t>
-        </is>
-      </c>
-      <c r="H4" s="11" t="n"/>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Quels conteneurs sont sur mon BL X ? / Visibilite BL sur OMNIO (a defaut d'un filtre OMNIO natif)</t>
+        </is>
+      </c>
       <c r="I4" s="11" t="n"/>
-      <c r="J4" s="7" t="inlineStr">
+      <c r="J4" s="11" t="n"/>
+      <c r="K4" s="7" t="inlineStr">
         <is>
           <t>A faire</t>
         </is>
       </c>
-      <c r="K4" s="11" t="n"/>
       <c r="L4" s="11" t="n"/>
+      <c r="M4" s="11" t="n"/>
     </row>
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="7" t="n">
@@ -1024,43 +1047,48 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
           <t>UNITS_BY_BOOKING_NUMBER</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="D5" s="10" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Units, filtre sur le champ Booking</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>Numero de booking</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>Numero conteneur, Statut, Date de gate-in, Navire, Voyage, Date de coupure (cut-off)</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Mes conteneurs export sont-ils bien receptionnes pour le booking Y ?</t>
         </is>
       </c>
-      <c r="H5" s="11" t="n"/>
       <c r="I5" s="11" t="n"/>
-      <c r="J5" s="7" t="inlineStr">
+      <c r="J5" s="11" t="n"/>
+      <c r="K5" s="7" t="inlineStr">
         <is>
           <t>A faire</t>
         </is>
       </c>
-      <c r="K5" s="11" t="n"/>
       <c r="L5" s="11" t="n"/>
+      <c r="M5" s="11" t="n"/>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="7" t="n">
@@ -1068,43 +1096,48 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
           <t>VESSEL_VISIT_BY_VOYAGE</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Moyenne-Haute</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>Vessel Visit / Vessel Screen</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>Numero de voyage (ou nom du navire + sens)</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>Nom du navire, Voyage, ETA, ATA, ETD, ATD, Statut de l'escale, Quai</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>Quand arrive le navire de mon conteneur ? / Est-il deja a quai ?</t>
         </is>
       </c>
-      <c r="H6" s="11" t="n"/>
       <c r="I6" s="11" t="n"/>
-      <c r="J6" s="7" t="inlineStr">
+      <c r="J6" s="11" t="n"/>
+      <c r="K6" s="7" t="inlineStr">
         <is>
           <t>A faire</t>
         </is>
       </c>
-      <c r="K6" s="11" t="n"/>
       <c r="L6" s="11" t="n"/>
+      <c r="M6" s="11" t="n"/>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="7" t="n">
@@ -1112,43 +1145,48 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
           <t>GATE_TRANSACTIONS_BY_UNIT</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="D7" s="13" t="inlineStr">
         <is>
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Gate Transactions / Truck Visit</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>Numero de conteneur</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Date/heure de transaction, Type (gate-in/gate-out), Numero de camion, Chauffeur, Statut de la transaction</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>Mon conteneur est-il deja sorti du terminal ?</t>
         </is>
       </c>
-      <c r="H7" s="11" t="n"/>
       <c r="I7" s="11" t="n"/>
-      <c r="J7" s="7" t="inlineStr">
+      <c r="J7" s="11" t="n"/>
+      <c r="K7" s="7" t="inlineStr">
         <is>
           <t>A faire</t>
         </is>
       </c>
-      <c r="K7" s="11" t="n"/>
       <c r="L7" s="11" t="n"/>
+      <c r="M7" s="11" t="n"/>
     </row>
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="7" t="n">
@@ -1156,43 +1194,48 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
           <t>UNIT_YARD_LOCATION</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>Basse (optionnel)</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>Yard Block / Yard View</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>Numero de conteneur</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>Bloc, Rangee, Baie, Niveau, Date d'entree en cour</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>Localisation physique precise (complement du filtre n°1)</t>
         </is>
       </c>
-      <c r="H8" s="11" t="n"/>
       <c r="I8" s="11" t="n"/>
-      <c r="J8" s="7" t="inlineStr">
+      <c r="J8" s="11" t="n"/>
+      <c r="K8" s="7" t="inlineStr">
         <is>
           <t>A faire</t>
         </is>
       </c>
-      <c r="K8" s="11" t="n"/>
       <c r="L8" s="11" t="n"/>
+      <c r="M8" s="11" t="n"/>
     </row>
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="7" t="n">
@@ -1200,43 +1243,48 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
           <t>UNIT_DAYS_IN_YARD</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>Basse-Moyenne</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>Units, avec calcul de duree (ou vue demurrage dediee)</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>Numero de conteneur</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>Date d'entree, Date du jour, Nombre de jours de sejour, Statut franchise (si calcule par Navis)</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>Depuis combien de temps mon conteneur est-il en cour ?</t>
         </is>
       </c>
-      <c r="H9" s="11" t="n"/>
       <c r="I9" s="11" t="n"/>
-      <c r="J9" s="7" t="inlineStr">
+      <c r="J9" s="11" t="n"/>
+      <c r="K9" s="7" t="inlineStr">
         <is>
           <t>A faire</t>
         </is>
       </c>
-      <c r="K9" s="11" t="n"/>
       <c r="L9" s="11" t="n"/>
+      <c r="M9" s="11" t="n"/>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="7" t="n">
@@ -1244,43 +1292,48 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
           <t>APPOINTMENT_STATUS</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>Ecran de rendez-vous/appointments du Gate (VBS)</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>Numero de conteneur, ou reference de rendez-vous, ou immatriculation camion</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>Reference du rendez-vous, Creneau (date/heure), Statut (confirme/annule/realise), Type d'operation (pickup/drop-off), Conteneur associe</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>Prise de rendez-vous / Annulation rendez-vous / Demande de creneau disponible / Indisponibilite VBS</t>
-        </is>
-      </c>
-      <c r="H10" s="11" t="n"/>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Prise de rendez-vous / Annulation rendez-vous / Demande de creneau disponible / Indisponibilite VBS (lecture de statut uniquement, jamais l'action de reserver/annuler)</t>
+        </is>
+      </c>
       <c r="I10" s="11" t="n"/>
-      <c r="J10" s="7" t="inlineStr">
+      <c r="J10" s="11" t="n"/>
+      <c r="K10" s="7" t="inlineStr">
         <is>
           <t>A faire</t>
         </is>
       </c>
-      <c r="K10" s="11" t="n"/>
       <c r="L10" s="11" t="n"/>
+      <c r="M10" s="11" t="n"/>
     </row>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="7" t="n">
@@ -1288,43 +1341,48 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
           <t>UNIT_VGM_STATUS</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>Units, colonnes VGM</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>Numero de conteneur</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Numero conteneur, VGM recu (oui/non), Poids VGM, Date de reception, Methode de pesee si tracee</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="H11" s="7" t="inlineStr">
         <is>
           <t>Probleme VGM</t>
         </is>
       </c>
-      <c r="H11" s="11" t="n"/>
       <c r="I11" s="11" t="n"/>
-      <c r="J11" s="7" t="inlineStr">
+      <c r="J11" s="11" t="n"/>
+      <c r="K11" s="7" t="inlineStr">
         <is>
           <t>A faire</t>
         </is>
       </c>
-      <c r="K11" s="11" t="n"/>
       <c r="L11" s="11" t="n"/>
+      <c r="M11" s="11" t="n"/>
     </row>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="7" t="n">
@@ -1332,43 +1390,48 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
           <t>EDI_MESSAGE_STATUS</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>Vue des messages EDI entrants (a confirmer si exposee en table)</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>Numero de BL ou de booking</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>Type de message (COPARN...), Date de reception, Statut (recu/rejete/en attente), Motif de rejet le cas echeant</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="H12" s="7" t="inlineStr">
         <is>
           <t>COPARN recu/non recu</t>
         </is>
       </c>
-      <c r="H12" s="11" t="n"/>
       <c r="I12" s="11" t="n"/>
-      <c r="J12" s="7" t="inlineStr">
+      <c r="J12" s="11" t="n"/>
+      <c r="K12" s="7" t="inlineStr">
         <is>
           <t>A faire</t>
         </is>
       </c>
-      <c r="K12" s="11" t="n"/>
       <c r="L12" s="11" t="n"/>
+      <c r="M12" s="11" t="n"/>
     </row>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="7" t="n">
@@ -1376,43 +1439,48 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
           <t>TRANSPORT_ORDER_STATUS</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>Transport Order (ASC Automated Equipment Database Interface)</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>Numero de conteneur, ou reference de mission</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>Reference mission, Type (pickup/dropoff/move), Statut (en attente/en cours/terminee/annulee), Equipement assigne</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>Mission conteneurs / Annulation mission / Assignation</t>
-        </is>
-      </c>
-      <c r="H13" s="11" t="n"/>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Mission conteneurs / Annulation mission (lecture de statut) / Assignation</t>
+        </is>
+      </c>
       <c r="I13" s="11" t="n"/>
-      <c r="J13" s="7" t="inlineStr">
+      <c r="J13" s="11" t="n"/>
+      <c r="K13" s="7" t="inlineStr">
         <is>
           <t>A faire</t>
         </is>
       </c>
-      <c r="K13" s="11" t="n"/>
       <c r="L13" s="11" t="n"/>
+      <c r="M13" s="11" t="n"/>
     </row>
     <row r="14" ht="60" customHeight="1">
       <c r="A14" s="7" t="n">
@@ -1420,48 +1488,53 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
           <t>TERMINAL_TRANSFER_STATUS</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr">
         <is>
           <t>Basse-Moyenne</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>A confirmer selon modelisation du transfert HINO/CIT</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>Numero de conteneur</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>Statut du transfert, Site d'origine, Site de destination, Date</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>Transfert conteneur HINO/CIT</t>
         </is>
       </c>
-      <c r="H14" s="11" t="n"/>
       <c r="I14" s="11" t="n"/>
-      <c r="J14" s="7" t="inlineStr">
+      <c r="J14" s="11" t="n"/>
+      <c r="K14" s="7" t="inlineStr">
         <is>
           <t>A faire</t>
         </is>
       </c>
-      <c r="K14" s="11" t="n"/>
       <c r="L14" s="11" t="n"/>
+      <c r="M14" s="11" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L14"/>
+  <autoFilter ref="A1:M14"/>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"A faire,En cours,Cree,Teste OK,Bloque"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1475,25 +1548,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Correspondance categories reelles -&gt; source de donnees</t>
+          <t>Correspondance categories reelles -&gt; Application / Filtre / Parametre</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>Source : REQUETE VBS.xlsx fourni par CIT (30 categories de requetes frequentes).</t>
+          <t>Source : REQUETE VBS.xlsx fourni par CIT (30 categories). Regle absolue : lecture seule. "Aucune (lecture impossible)" = action d'ecriture ou signalement d'incident, pas une donnee a lire.</t>
         </is>
       </c>
     </row>
@@ -1505,7 +1579,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Source proposee</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -1513,8 +1587,13 @@
           <t>Filtre</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="24" customHeight="1">
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Parametre</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Statut conteneurs</t>
@@ -1525,13 +1604,18 @@
           <t>Navis</t>
         </is>
       </c>
-      <c r="C5" s="19" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>#1 UNIT_STATUS_BY_NUMBER</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="24" customHeight="1">
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>N° conteneur</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
           <t>TC Introuvable</t>
@@ -1542,13 +1626,18 @@
           <t>Navis</t>
         </is>
       </c>
-      <c r="C6" s="19" t="inlineStr">
-        <is>
-          <t>#1</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>#1 UNIT_STATUS_BY_NUMBER</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>N° conteneur</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Position Conteneurs</t>
@@ -1559,13 +1648,18 @@
           <t>Navis</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
-        <is>
-          <t>#1 / #7</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="24" customHeight="1">
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>#1 / #7 UNIT_YARD_LOCATION</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>N° conteneur</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="26" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
           <t>TC innaccesible</t>
@@ -1573,16 +1667,21 @@
       </c>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>Navis (hold)</t>
-        </is>
-      </c>
-      <c r="C8" s="19" t="inlineStr">
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>#2 UNIT_HOLDS_BY_NUMBER</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>N° conteneur</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Debarquement conteneur dangereux</t>
@@ -1590,33 +1689,43 @@
       </c>
       <c r="B9" s="18" t="inlineStr">
         <is>
-          <t>Navis (statut + IMDG)</t>
-        </is>
-      </c>
-      <c r="C9" s="19" t="inlineStr">
-        <is>
-          <t>#1, colonnes etendues</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="17" t="inlineStr">
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>#1, colonnes IMDG</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>N° conteneur</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Visibilite BL sur OMNIO</t>
         </is>
       </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>Navis (OMNIO reflete Navis)</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="inlineStr">
-        <is>
-          <t>#3 UNITS_BY_BL_NUMBER</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>OMNIO (a defaut, Navis)</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Equivalent lecture BL cote OMNIO, sinon #3</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>N° de BL</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Nomination</t>
@@ -1627,13 +1736,18 @@
           <t>Navis</t>
         </is>
       </c>
-      <c r="C11" s="19" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>#4 UNITS_BY_BOOKING_NUMBER</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="24" customHeight="1">
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>N° de booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
       <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Situation Navire CIT</t>
@@ -1644,13 +1758,18 @@
           <t>Navis</t>
         </is>
       </c>
-      <c r="C12" s="19" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>#5 VESSEL_VISIT_BY_VOYAGE</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="24" customHeight="1">
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>N° de voyage</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Attente au chargement</t>
@@ -1658,16 +1777,21 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>Navis (gate)</t>
-        </is>
-      </c>
-      <c r="C13" s="19" t="inlineStr">
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
         <is>
           <t>#6 GATE_TRANSACTIONS_BY_UNIT</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="24" customHeight="1">
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>N° conteneur</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
       <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Embouteillage Sortie</t>
@@ -1675,16 +1799,21 @@
       </c>
       <c r="B14" s="18" t="inlineStr">
         <is>
-          <t>Navis (gate), si trace</t>
-        </is>
-      </c>
-      <c r="C14" s="19" t="inlineStr">
-        <is>
-          <t>#6</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="24" customHeight="1">
+          <t>Navis (si trace)</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>#6 GATE_TRANSACTIONS_BY_UNIT</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>N° conteneur</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Assignation</t>
@@ -1692,16 +1821,21 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>Navis (gate/mission)</t>
-        </is>
-      </c>
-      <c r="C15" s="19" t="inlineStr">
-        <is>
-          <t>#6 ou #12</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="24" customHeight="1">
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>#6 ou #12 TRANSPORT_ORDER_STATUS</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>N° conteneur / réf. mission</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
       <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Prise de rendez vous</t>
@@ -1712,13 +1846,18 @@
           <t>Navis (VBS)</t>
         </is>
       </c>
-      <c r="C16" s="19" t="inlineStr">
+      <c r="C16" s="18" t="inlineStr">
         <is>
           <t>#9 APPOINTMENT_STATUS</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="24" customHeight="1">
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>N° conteneur / réf. RDV</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Annulation rendez vous</t>
@@ -1729,13 +1868,18 @@
           <t>Navis (VBS)</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr">
-        <is>
-          <t>#9</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="24" customHeight="1">
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>#9 APPOINTMENT_STATUS (lecture du statut)</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>Réf. RDV</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
       <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Demande de creneau disponible</t>
@@ -1746,13 +1890,18 @@
           <t>Navis (VBS)</t>
         </is>
       </c>
-      <c r="C18" s="19" t="inlineStr">
-        <is>
-          <t>#9</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="24" customHeight="1">
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>#9 APPOINTMENT_STATUS (lecture des creneaux)</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Date / type d'operation</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1">
       <c r="A19" s="17" t="inlineStr">
         <is>
           <t>Indisponibilite VBS</t>
@@ -1760,16 +1909,21 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>Navis (VBS) - a confirmer</t>
-        </is>
-      </c>
-      <c r="C19" s="19" t="inlineStr">
-        <is>
-          <t>#9</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="24" customHeight="1">
+          <t>Navis (VBS), a confirmer</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>#9, si statut systeme expose</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="26" customHeight="1">
       <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Probleme VGM</t>
@@ -1780,13 +1934,18 @@
           <t>Navis</t>
         </is>
       </c>
-      <c r="C20" s="19" t="inlineStr">
+      <c r="C20" s="18" t="inlineStr">
         <is>
           <t>#10 UNIT_VGM_STATUS</t>
         </is>
       </c>
-    </row>
-    <row r="21" ht="24" customHeight="1">
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>N° conteneur</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
       <c r="A21" s="17" t="inlineStr">
         <is>
           <t>COPARN recu/non recu</t>
@@ -1797,13 +1956,18 @@
           <t>Navis (EDI)</t>
         </is>
       </c>
-      <c r="C21" s="19" t="inlineStr">
+      <c r="C21" s="18" t="inlineStr">
         <is>
           <t>#11 EDI_MESSAGE_STATUS</t>
         </is>
       </c>
-    </row>
-    <row r="22" ht="24" customHeight="1">
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>N° de BL/booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
       <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Mission conteneurs</t>
@@ -1811,16 +1975,21 @@
       </c>
       <c r="B22" s="18" t="inlineStr">
         <is>
-          <t>Navis (transport order)</t>
-        </is>
-      </c>
-      <c r="C22" s="19" t="inlineStr">
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
         <is>
           <t>#12 TRANSPORT_ORDER_STATUS</t>
         </is>
       </c>
-    </row>
-    <row r="23" ht="24" customHeight="1">
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>N° conteneur / réf. mission</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
           <t>Annulation mission</t>
@@ -1828,16 +1997,21 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>Navis (transport order)</t>
-        </is>
-      </c>
-      <c r="C23" s="19" t="inlineStr">
-        <is>
-          <t>#12</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="24" customHeight="1">
+          <t>Navis</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>#12 TRANSPORT_ORDER_STATUS (lecture du statut)</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>Réf. mission</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
       <c r="A24" s="17" t="inlineStr">
         <is>
           <t>Transfert conteneur HINO/CIT</t>
@@ -1845,169 +2019,219 @@
       </c>
       <c r="B24" s="18" t="inlineStr">
         <is>
-          <t>Navis, si trace</t>
-        </is>
-      </c>
-      <c r="C24" s="19" t="inlineStr">
+          <t>Navis (si trace)</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
         <is>
           <t>#13 TERMINAL_TRANSFER_STATUS</t>
         </is>
       </c>
-    </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="20" t="inlineStr">
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>N° conteneur</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="22" t="inlineStr">
         <is>
           <t>Creation Compte OMNIO</t>
         </is>
       </c>
-      <c r="B25" s="13" t="inlineStr">
-        <is>
-          <t>AMBIGU - action d'ecriture, pas une donnee a lire</t>
-        </is>
-      </c>
-      <c r="C25" s="21" t="inlineStr">
-        <is>
-          <t>A clarifier - voir note</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="20" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Aucune (lecture impossible)</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>Action d'ecriture — hors perimetre chatbot</t>
+        </is>
+      </c>
+      <c r="D25" s="23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="22" t="inlineStr">
         <is>
           <t>Activation compte OMNIO</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
-        <is>
-          <t>AMBIGU - idem</t>
-        </is>
-      </c>
-      <c r="C26" s="21" t="inlineStr">
-        <is>
-          <t>A clarifier</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="20" t="inlineStr">
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Aucune (lecture impossible)</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>Action d'ecriture — hors perimetre chatbot</t>
+        </is>
+      </c>
+      <c r="D26" s="23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1">
+      <c r="A27" s="22" t="inlineStr">
         <is>
           <t>Anomalie OMNIO</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
-        <is>
-          <t>AMBIGU - probablement incident technique</t>
-        </is>
-      </c>
-      <c r="C27" s="21" t="inlineStr">
-        <is>
-          <t>A clarifier</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="22" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Aucune (lecture impossible)</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Signalement d'incident — escalade humaine</t>
+        </is>
+      </c>
+      <c r="D27" s="23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="26" customHeight="1">
+      <c r="A28" s="24" t="inlineStr">
         <is>
           <t>Autorisation acces BL IES</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>Cote YABA (module IES)</t>
-        </is>
-      </c>
-      <c r="C28" s="23" t="inlineStr">
-        <is>
-          <t>Hors Navis</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="22" t="inlineStr">
+          <t>YABA</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>Module IES (decision metier)</t>
+        </is>
+      </c>
+      <c r="D28" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="26" customHeight="1">
+      <c r="A29" s="24" t="inlineStr">
         <is>
           <t>Actualisation BADT</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>Cote YABA (deja dans le ticket YABA, IMP-14)</t>
-        </is>
-      </c>
-      <c r="C29" s="23" t="inlineStr">
-        <is>
-          <t>Hors Navis</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="24" customHeight="1">
-      <c r="A30" s="22" t="inlineStr">
+          <t>YABA</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>Ticket YABA (IMP-14)</t>
+        </is>
+      </c>
+      <c r="D29" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="26" customHeight="1">
+      <c r="A30" s="24" t="inlineStr">
         <is>
           <t>BADT expire</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>Cote YABA</t>
-        </is>
-      </c>
-      <c r="C30" s="23" t="inlineStr">
-        <is>
-          <t>Hors Navis</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="24" customHeight="1">
-      <c r="A31" s="22" t="inlineStr">
+          <t>YABA</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>Ticket YABA</t>
+        </is>
+      </c>
+      <c r="D30" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="26" customHeight="1">
+      <c r="A31" s="24" t="inlineStr">
         <is>
           <t>Impression BEE</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
         <is>
-          <t>Cote YABA (deja dans le ticket YABA, EXP-03)</t>
-        </is>
-      </c>
-      <c r="C31" s="23" t="inlineStr">
-        <is>
-          <t>Hors Navis</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="24" customHeight="1">
+          <t>YABA</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Ticket YABA (EXP-03)</t>
+        </is>
+      </c>
+      <c r="D31" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="26" customHeight="1">
       <c r="A32" s="22" t="inlineStr">
         <is>
           <t>RTG en panne</t>
         </is>
       </c>
-      <c r="B32" s="14" t="inlineStr">
-        <is>
-          <t>Incident operationnel/equipement</t>
-        </is>
-      </c>
-      <c r="C32" s="23" t="inlineStr">
-        <is>
-          <t>Hors perimetre - escalade humaine</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="24" customHeight="1">
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>Aucune (lecture impossible)</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>Incident operationnel — escalade humaine</t>
+        </is>
+      </c>
+      <c r="D32" s="23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="26" customHeight="1">
       <c r="A33" s="22" t="inlineStr">
         <is>
           <t>Probleme de reseau</t>
         </is>
       </c>
-      <c r="B33" s="14" t="inlineStr">
-        <is>
-          <t>Incident IT</t>
-        </is>
-      </c>
-      <c r="C33" s="23" t="inlineStr">
-        <is>
-          <t>Hors perimetre - escalade humaine</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="24" customHeight="1">
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>Aucune (lecture impossible)</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>Incident IT — escalade humaine</t>
+        </is>
+      </c>
+      <c r="D33" s="23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1">
       <c r="A34" s="17" t="inlineStr">
         <is>
           <t>Autre</t>
@@ -2015,20 +2239,25 @@
       </c>
       <c r="B34" s="18" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C34" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C34" s="18" t="inlineStr">
         <is>
           <t>Toujours escalade humaine (IA-03)</t>
         </is>
       </c>
+      <c r="D34" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:C34"/>
+  <autoFilter ref="A4:D34"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2055,7 +2284,7 @@
       </c>
     </row>
     <row r="3" ht="50" customHeight="1">
-      <c r="A3" s="24" t="inlineStr">
+      <c r="A3" s="26" t="inlineStr">
         <is>
           <t>Facturation / paiement</t>
         </is>
@@ -2067,7 +2296,7 @@
       </c>
     </row>
     <row r="4" ht="50" customHeight="1">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="26" t="inlineStr">
         <is>
           <t>Toute action en ecriture (holds, confirmations, creation/activation de compte...)</t>
         </is>
@@ -2079,7 +2308,7 @@
       </c>
     </row>
     <row r="5" ht="50" customHeight="1">
-      <c r="A5" s="24" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>BADT / BEE (actualisation, expiration, impression)</t>
         </is>
@@ -2091,7 +2320,7 @@
       </c>
     </row>
     <row r="6" ht="50" customHeight="1">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="A6" s="26" t="inlineStr">
         <is>
           <t>RTG en panne, Probleme de reseau</t>
         </is>

</xml_diff>

<commit_message>
docs(navis): en-tetes de colonnes du classeur filtres en anglais
</commit_message>
<xml_diff>
--- a/docs/99-filtres-navis-a-creer.xlsx
+++ b/docs/99-filtres-navis-a-creer.xlsx
@@ -662,17 +662,17 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Champ</t>
+          <t>Field</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Indication / exemple</t>
+          <t>Hint / example</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Valeur reelle (a remplir)</t>
+          <t>Actual value (to fill in)</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Nom du compte</t>
+          <t>Account name</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Filtres qu'il doit voir</t>
+          <t>Filters it must see</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>N°</t>
+          <t>No.</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
@@ -840,57 +840,57 @@
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>Nom du filtre (propose)</t>
+          <t>Filter name (proposed)</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>Priorite</t>
+          <t>Priority</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>Ecran N4 source</t>
+          <t>Source N4 screen</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>Parametre attendu</t>
+          <t>Expected parameter</t>
         </is>
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
-          <t>Colonnes a inclure</t>
+          <t>Columns to include</t>
         </is>
       </c>
       <c r="H1" s="5" t="inlineStr">
         <is>
-          <t>Question client couverte</t>
+          <t>Customer question covered</t>
         </is>
       </c>
       <c r="I1" s="5" t="inlineStr">
         <is>
-          <t>Nom reel enregistre (si different)</t>
+          <t>Actual saved name (if different)</t>
         </is>
       </c>
       <c r="J1" s="5" t="inlineStr">
         <is>
-          <t>Nom reel du champ parametre</t>
+          <t>Actual parameter field name</t>
         </is>
       </c>
       <c r="K1" s="5" t="inlineStr">
         <is>
-          <t>Statut</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="L1" s="5" t="inlineStr">
         <is>
-          <t>Date de creation</t>
+          <t>Creation date</t>
         </is>
       </c>
       <c r="M1" s="5" t="inlineStr">
         <is>
-          <t>Commentaire / testeur</t>
+          <t>Comment / tester</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Categorie reelle (FAQ)</t>
+          <t>Real category (FAQ)</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1584,12 +1584,12 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Filtre</t>
+          <t>Filter</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Parametre</t>
+          <t>Parameter</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(navis): contenu de la colonne Columns to include en anglais
</commit_message>
<xml_diff>
--- a/docs/99-filtres-navis-a-creer.xlsx
+++ b/docs/99-filtres-navis-a-creer.xlsx
@@ -925,7 +925,7 @@
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
-          <t>Numero conteneur, Statut/Category, Emplacement (bloc/rangee/niveau), Navire, Voyage, Sens (Import/Export), Date de dechargement (ou gate-in export), Ligne maritime</t>
+          <t>Container number, Status/Category, Location (block/row/tier), Vessel, Voyage, Direction (Import/Export), Discharge date (or export gate-in), Shipping line</t>
         </is>
       </c>
       <c r="H2" s="7" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>Numero conteneur, Type de hold (douane, facturation, ligne...), Statut du hold (actif/leve), Raison, Date de pose</t>
+          <t>Container number, Hold type (customs, billing, line...), Hold status (active/released), Reason, Date placed</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>Numero conteneur, Statut, Emplacement, Poids, Taille/Type</t>
+          <t>Container number, Status, Location, Weight, Size/Type</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>Numero conteneur, Statut, Date de gate-in, Navire, Voyage, Date de coupure (cut-off)</t>
+          <t>Container number, Status, Gate-in date, Vessel, Voyage, Cut-off date</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Nom du navire, Voyage, ETA, ATA, ETD, ATD, Statut de l'escale, Quai</t>
+          <t>Vessel name, Voyage, ETA, ATA, ETD, ATD, Call status, Berth</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Date/heure de transaction, Type (gate-in/gate-out), Numero de camion, Chauffeur, Statut de la transaction</t>
+          <t>Transaction date/time, Type (gate-in/gate-out), Truck number, Driver, Transaction status</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Bloc, Rangee, Baie, Niveau, Date d'entree en cour</t>
+          <t>Block, Row, Bay, Tier, Yard-in date</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Date d'entree, Date du jour, Nombre de jours de sejour, Statut franchise (si calcule par Navis)</t>
+          <t>Entry date, Current date, Number of dwell days, Free-time status (if computed by Navis)</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Reference du rendez-vous, Creneau (date/heure), Statut (confirme/annule/realise), Type d'operation (pickup/drop-off), Conteneur associe</t>
+          <t>Appointment reference, Slot (date/time), Status (confirmed/cancelled/completed), Operation type (pickup/drop-off), Associated container</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Numero conteneur, VGM recu (oui/non), Poids VGM, Date de reception, Methode de pesee si tracee</t>
+          <t>Container number, VGM received (yes/no), VGM weight, Received date, Weighing method if tracked</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -1415,7 +1415,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Type de message (COPARN...), Date de reception, Statut (recu/rejete/en attente), Motif de rejet le cas echeant</t>
+          <t>Message type (COPARN...), Received date, Status (received/rejected/pending), Rejection reason if any</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Reference mission, Type (pickup/dropoff/move), Statut (en attente/en cours/terminee/annulee), Equipement assigne</t>
+          <t>Order reference, Type (pickup/dropoff/move), Status (pending/in progress/completed/cancelled), Assigned equipment</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Statut du transfert, Site d'origine, Site de destination, Date</t>
+          <t>Transfer status, Origin site, Destination site, Date</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">

</xml_diff>